<commit_message>
auto: session 2026-09-14 11:16
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/mau-4.xlsx
+++ b/templates/mau-4.xlsx
@@ -912,7 +912,7 @@
         <xdr:cNvPr id="1" name="image1.png" descr="Image 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:id="{7b3a0b5b-92b4-4bd1-b9d8-b5c6fd9062a4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7b3a0b5b-92b4-4bd1-b9d8-b5c6fd9062a4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -950,7 +950,7 @@
         <xdr:cNvPr id="2" name="image2.png" descr="Stamp">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:id="{2ed2edcb-4787-4261-a784-43f07b2ab983}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2ed2edcb-4787-4261-a784-43f07b2ab983}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>

</xml_diff>